<commit_message>
feat(regtab): add multi-model family support; expand effecttab options
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_effecttab.xlsx
+++ b/tabtools/demo/demo_effecttab.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="132" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="132" uniqueCount="40">
   <si>
     <t>Table 6. Average Treatment Effect on CV Events (IPW)</t>
   </si>
@@ -42,10 +42,10 @@
     <t>95% CI</t>
   </si>
   <si>
-    <t>(-0.008446304802640723, 0.02268258272179105)</t>
+    <t>(-0.01, 0.02)</t>
   </si>
   <si>
-    <t>(0.33754377991200185, 0.35729196506214417)</t>
+    <t>(0.34, 0.36)</t>
   </si>
   <si>
     <t>p-value</t>
@@ -66,12 +66,6 @@
     <t>AIPW</t>
   </si>
   <si>
-    <t>(-0.008446918773028899, 0.022681791080266387)</t>
-  </si>
-  <si>
-    <t>(0.33754598917417244, 0.35729440629461096)</t>
-  </si>
-  <si>
     <t>IPW = inverse probability weighting. AIPW = augmented IPW (doubly robust).</t>
   </si>
   <si>
@@ -87,10 +81,7 @@
     <t>Pr(CV Event)</t>
   </si>
   <si>
-    <t>(0.3373043379056112, 0.357042678371268)</t>
-  </si>
-  <si>
-    <t>(0.3419777255620122, 0.3660365568699804)</t>
+    <t>(0.34, 0.37)</t>
   </si>
   <si>
     <t>Table 9. Average Marginal Effects on CV Event Risk</t>
@@ -120,19 +111,13 @@
     <t>0.02</t>
   </si>
   <si>
-    <t>(-0.008684430040083813, 0.02237140219063296)</t>
+    <t>(0.00, 0.00)</t>
   </si>
   <si>
-    <t>(3.287866087374632e-05, 0.0011785093697413455)</t>
+    <t>(0.01, 0.04)</t>
   </si>
   <si>
-    <t>(-0.01402975513266309, 0.017090394200780498)</t>
-  </si>
-  <si>
-    <t>(0.00563916610651144, 0.036633624833529194)</t>
-  </si>
-  <si>
-    <t>(-0.016860214198001204, 0.014192203531617365)</t>
+    <t>(-0.02, 0.01)</t>
   </si>
   <si>
     <t>0.39</t>
@@ -7998,7 +7983,7 @@
     <col min="1" max="1" width="1.7109375" style="2" customWidth="true"/>
     <col min="2" max="2" width="16.7109375" style="3" customWidth="true"/>
     <col min="3" max="3" width="8.7109375" style="4" customWidth="true"/>
-    <col min="4" max="4" width="34.7109375" style="5" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="5" customWidth="true"/>
     <col min="5" max="5" width="8.7109375" style="6" customWidth="true"/>
   </cols>
   <sheetData>
@@ -8104,8 +8089,8 @@
     <col min="2" max="2" width="16.7109375" style="96" customWidth="true"/>
     <col min="3" max="3" width="8.7109375" style="97" customWidth="true"/>
     <col min="6" max="6" width="8.7109375" style="98" customWidth="true"/>
-    <col min="4" max="4" width="34.7109375" style="99" customWidth="true"/>
-    <col min="7" max="7" width="34.7109375" style="100" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="99" customWidth="true"/>
+    <col min="7" max="7" width="16.7109375" style="100" customWidth="true"/>
     <col min="5" max="5" width="8.7109375" style="101" customWidth="true"/>
     <col min="8" max="8" width="8.7109375" style="102" customWidth="true"/>
   </cols>
@@ -8208,7 +8193,7 @@
         <v>5</v>
       </c>
       <c r="G4" s="242" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H4" s="243" t="s">
         <v>11</v>
@@ -8234,7 +8219,7 @@
         <v>6</v>
       </c>
       <c r="G5" s="248" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H5" s="249" t="s">
         <v>12</v>
@@ -8242,7 +8227,7 @@
     </row>
     <row r="6">
       <c r="B6" s="254" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" s="0"/>
       <c r="D6" s="0"/>
@@ -8269,13 +8254,13 @@
     <col min="1" max="1" width="1.7109375" style="256" customWidth="true"/>
     <col min="2" max="2" width="13.7109375" style="257" customWidth="true"/>
     <col min="3" max="3" width="13.7109375" style="258" customWidth="true"/>
-    <col min="4" max="4" width="34.7109375" style="259" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="259" customWidth="true"/>
     <col min="5" max="5" width="8.7109375" style="260" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" s="255" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="294" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B1" s="286" t="s">
         <v>1</v>
@@ -8315,7 +8300,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="323" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D3" s="324" t="s">
         <v>7</v>
@@ -8329,13 +8314,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="340" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C4" s="342" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="343" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="E4" s="344" t="s">
         <v>12</v>
@@ -8346,13 +8331,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="341" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="345" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="346" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E5" s="347" t="s">
         <v>12</v>
@@ -8374,13 +8359,13 @@
     <col min="1" max="1" width="1.7109375" style="349" customWidth="true"/>
     <col min="2" max="2" width="28.7109375" style="350" customWidth="true"/>
     <col min="3" max="3" width="8.7109375" style="351" customWidth="true"/>
-    <col min="4" max="4" width="34.7109375" style="352" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="352" customWidth="true"/>
     <col min="5" max="5" width="8.7109375" style="353" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" s="348" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="402" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B1" s="394" t="s">
         <v>1</v>
@@ -8420,7 +8405,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="434" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D3" s="435" t="s">
         <v>7</v>
@@ -8434,16 +8419,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="457" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C4" s="462" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="463" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="464" t="s">
         <v>34</v>
-      </c>
-      <c r="E4" s="464" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -8451,16 +8436,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="458" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C5" s="465" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D5" s="466" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="467" t="s">
         <v>35</v>
-      </c>
-      <c r="E5" s="467" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="6">
@@ -8468,16 +8453,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="459" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C6" s="468" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D6" s="469" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="470" t="s">
         <v>36</v>
-      </c>
-      <c r="E6" s="470" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="7">
@@ -8485,16 +8470,16 @@
         <v>1</v>
       </c>
       <c r="B7" s="460" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C7" s="471" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D7" s="472" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="473" t="s">
         <v>37</v>
-      </c>
-      <c r="E7" s="473" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -8502,21 +8487,21 @@
         <v>1</v>
       </c>
       <c r="B8" s="461" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C8" s="474" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D8" s="475" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="476" t="s">
         <v>38</v>
-      </c>
-      <c r="E8" s="476" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="481" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C9" s="0"/>
       <c r="D9" s="0"/>

</xml_diff>

<commit_message>
feat(tabtools): add markdown export support across all table commands
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_effecttab.xlsx
+++ b/tabtools/demo/demo_effecttab.xlsx
@@ -142,7 +142,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="640">
+  <fonts count="662">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -671,6 +687,22 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -1566,6 +1598,22 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -2079,6 +2127,46 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2906,7 +2994,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="482">
+  <borders count="504">
     <border>
       <left/>
       <right/>
@@ -2920,6 +3008,34 @@
     <border/>
     <border/>
     <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -4079,6 +4195,34 @@
     </border>
     <border>
       <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
       <right style="thin"/>
       <top style="none"/>
       <bottom style="none"/>
@@ -4960,6 +5104,34 @@
     </border>
     <border>
       <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
       <right style="thin"/>
       <top style="none"/>
       <bottom style="none"/>
@@ -5680,6 +5852,76 @@
     </border>
     <border>
       <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
       <right style="thin"/>
       <top style="none"/>
       <bottom style="none"/>
@@ -6123,7 +6365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="482">
+  <cellXfs count="504">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -6131,252 +6373,252 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="22" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="23" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="25" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="26" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="27" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="28" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="29" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="30" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="31" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="32" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="35" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="36" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="37" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="38" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="22" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="23" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="24" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="25" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="26" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="27" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="28" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="29" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="30" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="31" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="32" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="35" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="36" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="37" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="38" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="39" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="41" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="42" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="63" fillId="0" borderId="39" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="67" fillId="0" borderId="43" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="65" fillId="0" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="67" fillId="0" borderId="41" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="42" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="43" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="73" fillId="0" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="45" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="45" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="0" borderId="46" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="75" fillId="0" borderId="47" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="48" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="0" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="75" fillId="0" borderId="46" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="50" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="47" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="80" fillId="0" borderId="51" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="48" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="52" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="82" fillId="0" borderId="53" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="79" fillId="0" borderId="50" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="80" fillId="0" borderId="51" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="52" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="82" fillId="0" borderId="53" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="83" fillId="0" borderId="54" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="85" fillId="0" borderId="55" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="84" fillId="0" borderId="55" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="86" fillId="0" borderId="56" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="56" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="86" fillId="0" borderId="57" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="87" fillId="0" borderId="58" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="89" fillId="0" borderId="59" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="90" fillId="0" borderId="60" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="57" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="88" fillId="0" borderId="58" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="61" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="92" fillId="0" borderId="62" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="89" fillId="0" borderId="59" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="90" fillId="0" borderId="60" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="91" fillId="0" borderId="61" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="92" fillId="0" borderId="62" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="93" fillId="0" borderId="63" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="64" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="65" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="96" fillId="0" borderId="66" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="63" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="94" fillId="0" borderId="64" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="95" fillId="0" borderId="65" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="66" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="0" fontId="97" fillId="0" borderId="67" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="98" fillId="0" borderId="68" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="99" fillId="0" borderId="69" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -6392,27 +6634,27 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="102" fillId="0" borderId="72" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="103" fillId="0" borderId="73" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="104" fillId="0" borderId="74" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="105" fillId="0" borderId="75" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="106" fillId="0" borderId="76" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="107" fillId="0" borderId="77" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="108" fillId="0" borderId="78" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -6448,27 +6690,27 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="116" fillId="0" borderId="86" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="117" fillId="0" borderId="87" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="118" fillId="0" borderId="88" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="119" fillId="0" borderId="89" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="120" fillId="0" borderId="90" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="121" fillId="0" borderId="91" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="122" fillId="0" borderId="92" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -6479,305 +6721,305 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="97" xfId="0"/>
+    <xf numFmtId="0" fontId="124" fillId="0" borderId="94" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="125" fillId="0" borderId="95" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="126" fillId="0" borderId="96" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="127" fillId="0" borderId="97" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="98" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="99" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="100" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="101" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="102" xfId="0"/>
-    <xf numFmtId="0" fontId="125" fillId="0" borderId="103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="127" fillId="0" borderId="104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="129" fillId="0" borderId="105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="131" fillId="0" borderId="106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="133" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="135" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="137" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="139" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="141" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="143" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="145" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="147" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="149" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="151" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="153" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="155" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="157" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="159" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="161" fillId="0" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="163" fillId="0" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="165" fillId="0" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="167" fillId="0" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="169" fillId="0" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="171" fillId="0" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="173" fillId="0" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="175" fillId="0" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="177" fillId="0" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="179" fillId="0" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="181" fillId="0" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="183" fillId="0" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="185" fillId="0" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="187" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="189" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="191" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="193" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="195" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="197" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="199" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="201" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="203" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="205" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="207" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="209" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="211" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="213" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="215" fillId="0" borderId="148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="217" fillId="0" borderId="149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="219" fillId="0" borderId="150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="220" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="103" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="104" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="105" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="106" xfId="0"/>
+    <xf numFmtId="0" fontId="128" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="221" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="129" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="130" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="131" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="133" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="135" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="137" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="139" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="141" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="143" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="145" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="147" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="149" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="151" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="153" fillId="0" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="155" fillId="0" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="157" fillId="0" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="159" fillId="0" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="161" fillId="0" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="163" fillId="0" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="165" fillId="0" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="167" fillId="0" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="169" fillId="0" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="171" fillId="0" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="173" fillId="0" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="175" fillId="0" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="177" fillId="0" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="179" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="181" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="183" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="185" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="187" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="189" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="191" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="193" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="195" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="197" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="199" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="201" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="203" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="205" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="207" fillId="0" borderId="148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="209" fillId="0" borderId="149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="211" fillId="0" borderId="150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="213" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="215" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="217" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="219" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="221" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="223" fillId="0" borderId="156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="225" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="227" fillId="0" borderId="158" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="228" fillId="0" borderId="159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="229" fillId="0" borderId="160" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="222" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="230" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="224" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="232" fillId="0" borderId="162" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="226" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="228" fillId="0" borderId="156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="230" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="232" fillId="0" borderId="158" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="234" fillId="0" borderId="159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="236" fillId="0" borderId="160" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="238" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="239" fillId="0" borderId="162" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="234" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="236" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="238" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="240" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="242" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="244" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="246" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="247" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="240" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="248" fillId="0" borderId="171" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="241" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="249" fillId="0" borderId="172" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="242" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="250" fillId="0" borderId="173" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="243" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="251" fillId="0" borderId="174" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="244" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="252" fillId="0" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="245" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="246" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="247" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="248" fillId="0" borderId="171" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="249" fillId="0" borderId="172" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="250" fillId="0" borderId="173" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="251" fillId="0" borderId="174" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="252" fillId="0" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="253" fillId="0" borderId="176" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -6788,120 +7030,120 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="256" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="255" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="257" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="256" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="257" fillId="0" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="258" fillId="0" borderId="181" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="259" fillId="0" borderId="182" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="260" fillId="0" borderId="183" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="261" fillId="0" borderId="184" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="262" fillId="0" borderId="185" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="264" fillId="0" borderId="186" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="265" fillId="0" borderId="187" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="258" fillId="0" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="259" fillId="0" borderId="181" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="266" fillId="0" borderId="188" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="267" fillId="0" borderId="189" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="260" fillId="0" borderId="182" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="261" fillId="0" borderId="183" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="262" fillId="0" borderId="184" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="268" fillId="0" borderId="190" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="269" fillId="0" borderId="191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="270" fillId="0" borderId="192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="263" fillId="0" borderId="185" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="271" fillId="0" borderId="193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="186" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="273" fillId="0" borderId="194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="266" fillId="0" borderId="187" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="274" fillId="0" borderId="195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="267" fillId="0" borderId="188" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="268" fillId="0" borderId="189" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="275" fillId="0" borderId="196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="276" fillId="0" borderId="197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="269" fillId="0" borderId="190" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="270" fillId="0" borderId="191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="271" fillId="0" borderId="192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="272" fillId="0" borderId="193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="277" fillId="0" borderId="198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="278" fillId="0" borderId="199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="279" fillId="0" borderId="200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="280" fillId="0" borderId="201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="273" fillId="0" borderId="194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="274" fillId="0" borderId="195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="275" fillId="0" borderId="196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="281" fillId="0" borderId="202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="282" fillId="0" borderId="203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="283" fillId="0" borderId="204" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="276" fillId="0" borderId="197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="277" fillId="0" borderId="198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="278" fillId="0" borderId="199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="279" fillId="0" borderId="200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="280" fillId="0" borderId="201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="281" fillId="0" borderId="202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="282" fillId="0" borderId="203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="283" fillId="0" borderId="204" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="0" fontId="284" fillId="0" borderId="205" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="285" fillId="0" borderId="206" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="286" fillId="0" borderId="207" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -6925,39 +7167,39 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="291" fillId="0" borderId="212" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="292" fillId="0" borderId="213" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="293" fillId="0" borderId="214" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="294" fillId="0" borderId="215" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="295" fillId="0" borderId="216" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="296" fillId="0" borderId="217" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="297" fillId="0" borderId="218" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="298" fillId="0" borderId="219" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="299" fillId="0" borderId="220" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="300" fillId="0" borderId="221" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -6973,7 +7215,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="303" fillId="0" borderId="224" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="304" fillId="0" borderId="225" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7000,345 +7242,345 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="310" fillId="2" borderId="231" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="311" fillId="3" borderId="232" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="312" fillId="4" borderId="233" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="313" fillId="5" borderId="234" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="314" fillId="6" borderId="235" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="315" fillId="7" borderId="236" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="316" fillId="8" borderId="237" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="310" fillId="0" borderId="231" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="311" fillId="0" borderId="232" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="312" fillId="0" borderId="233" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="313" fillId="0" borderId="234" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="314" fillId="0" borderId="235" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="315" fillId="0" borderId="236" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="316" fillId="0" borderId="237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="317" fillId="0" borderId="238" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="318" fillId="2" borderId="239" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="319" fillId="3" borderId="240" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="320" fillId="4" borderId="241" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="321" fillId="5" borderId="242" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="322" fillId="6" borderId="243" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="323" fillId="7" borderId="244" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="324" fillId="8" borderId="245" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="325" fillId="0" borderId="246" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="318" fillId="0" borderId="239" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="326" fillId="0" borderId="247" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="319" fillId="0" borderId="240" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="327" fillId="0" borderId="248" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="320" fillId="0" borderId="241" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="328" fillId="0" borderId="249" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="321" fillId="0" borderId="242" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="329" fillId="0" borderId="250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="322" fillId="0" borderId="243" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="330" fillId="0" borderId="251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="323" fillId="9" borderId="244" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="331" fillId="9" borderId="252" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="324" fillId="10" borderId="245" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="332" fillId="10" borderId="253" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="325" fillId="11" borderId="246" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="333" fillId="11" borderId="254" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="326" fillId="12" borderId="247" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="334" fillId="12" borderId="255" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="327" fillId="13" borderId="248" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="335" fillId="13" borderId="256" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="328" fillId="14" borderId="249" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="336" fillId="14" borderId="257" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="329" fillId="0" borderId="250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="337" fillId="0" borderId="258" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="330" fillId="0" borderId="251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="338" fillId="0" borderId="259" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="331" fillId="0" borderId="252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="339" fillId="0" borderId="260" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="333" fillId="0" borderId="253" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="341" fillId="0" borderId="261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="335" fillId="0" borderId="254" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="343" fillId="0" borderId="262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="255" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="256" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="257" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="258" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="259" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="260" xfId="0"/>
-    <xf numFmtId="0" fontId="337" fillId="0" borderId="261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="339" fillId="0" borderId="262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="341" fillId="0" borderId="263" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="343" fillId="0" borderId="264" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="345" fillId="0" borderId="265" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="347" fillId="0" borderId="266" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="349" fillId="0" borderId="267" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="351" fillId="0" borderId="268" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="353" fillId="0" borderId="269" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="355" fillId="0" borderId="270" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="357" fillId="0" borderId="271" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="359" fillId="0" borderId="272" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="361" fillId="0" borderId="273" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="363" fillId="0" borderId="274" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="365" fillId="0" borderId="275" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="367" fillId="0" borderId="276" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="369" fillId="0" borderId="277" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="371" fillId="0" borderId="278" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="373" fillId="0" borderId="279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="375" fillId="0" borderId="280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="377" fillId="0" borderId="281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="379" fillId="0" borderId="282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="381" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="383" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="385" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="387" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="389" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="391" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="393" fillId="0" borderId="289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="395" fillId="0" borderId="290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="396" fillId="0" borderId="291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="263" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="264" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="265" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="266" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="267" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="268" xfId="0"/>
+    <xf numFmtId="0" fontId="344" fillId="0" borderId="269" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="397" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="345" fillId="0" borderId="270" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="346" fillId="0" borderId="271" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="347" fillId="0" borderId="272" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="349" fillId="0" borderId="273" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="351" fillId="0" borderId="274" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="353" fillId="0" borderId="275" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="355" fillId="0" borderId="276" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="357" fillId="0" borderId="277" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="359" fillId="0" borderId="278" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="361" fillId="0" borderId="279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="363" fillId="0" borderId="280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="365" fillId="0" borderId="281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="367" fillId="0" borderId="282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="369" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="371" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="373" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="375" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="377" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="379" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="381" fillId="0" borderId="289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="383" fillId="0" borderId="290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="385" fillId="0" borderId="291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="387" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="389" fillId="0" borderId="293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="391" fillId="0" borderId="294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="393" fillId="0" borderId="295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="395" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="397" fillId="0" borderId="297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="399" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="401" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="403" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="405" fillId="0" borderId="301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="407" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="408" fillId="0" borderId="303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="409" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="398" fillId="0" borderId="293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="410" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="400" fillId="0" borderId="294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="412" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="402" fillId="0" borderId="295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="404" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="406" fillId="0" borderId="297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="408" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="409" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="414" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="416" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="418" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="420" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="421" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="410" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="422" fillId="0" borderId="312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="411" fillId="0" borderId="301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="423" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="412" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="424" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="413" fillId="0" borderId="303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="425" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="414" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="426" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="415" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="427" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="416" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="428" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="417" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="429" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="418" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="420" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="421" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="422" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="423" fillId="0" borderId="312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="424" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="425" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="426" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="427" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="428" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="429" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="430" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="431" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="430" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7347,11 +7589,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="433" fillId="0" borderId="322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="434" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="435" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7359,7 +7601,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="436" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="437" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7371,7 +7613,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="439" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="440" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7387,15 +7629,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="443" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="444" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="445" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="446" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7403,405 +7645,405 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="447" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="448" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="449" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="450" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="451" fillId="0" borderId="340" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="452" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="453" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="454" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="451" fillId="0" borderId="340" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="452" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="453" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="455" fillId="0" borderId="344" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="456" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="457" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="458" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="459" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="460" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="461" fillId="0" borderId="350" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="462" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="463" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="464" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="465" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="454" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="466" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="455" fillId="0" borderId="344" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="467" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="456" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="468" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="457" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="469" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="458" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="470" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="348" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="349" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="350" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="351" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="352" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="353" xfId="0"/>
-    <xf numFmtId="0" fontId="460" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="462" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="464" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="466" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="468" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="470" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="472" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="474" fillId="0" borderId="361" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="476" fillId="0" borderId="362" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="478" fillId="0" borderId="363" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="480" fillId="0" borderId="364" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="482" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="484" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="486" fillId="0" borderId="367" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="488" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="490" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="492" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="494" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="496" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="498" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="500" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="502" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="504" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="506" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="508" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="510" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="512" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="514" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="516" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="518" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="520" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="522" fillId="0" borderId="385" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="524" fillId="0" borderId="386" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="526" fillId="0" borderId="387" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="528" fillId="0" borderId="388" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="530" fillId="0" borderId="389" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="532" fillId="0" borderId="390" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="534" fillId="0" borderId="391" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="536" fillId="0" borderId="392" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="538" fillId="0" borderId="393" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="540" fillId="0" borderId="394" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="542" fillId="0" borderId="395" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="544" fillId="0" borderId="396" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="546" fillId="0" borderId="397" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="548" fillId="0" borderId="398" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="549" fillId="0" borderId="399" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="360" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="361" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="362" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="363" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="364" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="365" xfId="0"/>
+    <xf numFmtId="0" fontId="471" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="550" fillId="0" borderId="400" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="472" fillId="0" borderId="367" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="473" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="474" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="475" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="476" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="477" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="478" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="479" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="480" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="482" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="484" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="486" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="488" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="490" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="492" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="494" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="496" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="498" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="500" fillId="0" borderId="385" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="502" fillId="0" borderId="386" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="504" fillId="0" borderId="387" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="506" fillId="0" borderId="388" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="508" fillId="0" borderId="389" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="510" fillId="0" borderId="390" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="512" fillId="0" borderId="391" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="514" fillId="0" borderId="392" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="516" fillId="0" borderId="393" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="518" fillId="0" borderId="394" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="520" fillId="0" borderId="395" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="522" fillId="0" borderId="396" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="524" fillId="0" borderId="397" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="526" fillId="0" borderId="398" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="528" fillId="0" borderId="399" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="530" fillId="0" borderId="400" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="532" fillId="0" borderId="401" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="534" fillId="0" borderId="402" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="536" fillId="0" borderId="403" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="538" fillId="0" borderId="404" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="540" fillId="0" borderId="405" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="542" fillId="0" borderId="406" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="544" fillId="0" borderId="407" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="546" fillId="0" borderId="408" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="548" fillId="0" borderId="409" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="550" fillId="0" borderId="410" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="552" fillId="0" borderId="411" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="554" fillId="0" borderId="412" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="556" fillId="0" borderId="413" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="558" fillId="0" borderId="414" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="560" fillId="0" borderId="415" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="562" fillId="0" borderId="416" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="564" fillId="0" borderId="417" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="566" fillId="0" borderId="418" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="568" fillId="0" borderId="419" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="570" fillId="0" borderId="420" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="571" fillId="0" borderId="421" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="572" fillId="0" borderId="422" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="551" fillId="0" borderId="401" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="573" fillId="0" borderId="423" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="553" fillId="0" borderId="402" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="575" fillId="0" borderId="424" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="555" fillId="0" borderId="403" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="557" fillId="0" borderId="404" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="559" fillId="0" borderId="405" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="561" fillId="0" borderId="406" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="562" fillId="0" borderId="407" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="577" fillId="0" borderId="425" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="579" fillId="0" borderId="426" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="581" fillId="0" borderId="427" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="583" fillId="0" borderId="428" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="584" fillId="0" borderId="429" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="563" fillId="0" borderId="408" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="585" fillId="0" borderId="430" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="564" fillId="0" borderId="409" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="586" fillId="0" borderId="431" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="565" fillId="0" borderId="410" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="587" fillId="0" borderId="432" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="566" fillId="0" borderId="411" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="588" fillId="0" borderId="433" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="567" fillId="0" borderId="412" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="589" fillId="0" borderId="434" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="568" fillId="0" borderId="413" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="590" fillId="0" borderId="435" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="569" fillId="0" borderId="414" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="591" fillId="0" borderId="436" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="570" fillId="0" borderId="415" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="592" fillId="0" borderId="437" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="571" fillId="0" borderId="416" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="593" fillId="0" borderId="438" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="573" fillId="0" borderId="417" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="595" fillId="0" borderId="439" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="574" fillId="0" borderId="418" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="596" fillId="0" borderId="440" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="575" fillId="0" borderId="419" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="576" fillId="0" borderId="420" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="577" fillId="0" borderId="421" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="578" fillId="0" borderId="422" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="579" fillId="0" borderId="423" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="580" fillId="0" borderId="424" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="581" fillId="0" borderId="425" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="582" fillId="0" borderId="426" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="583" fillId="0" borderId="427" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="584" fillId="0" borderId="428" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="585" fillId="0" borderId="429" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="586" fillId="0" borderId="430" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="587" fillId="0" borderId="431" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="588" fillId="0" borderId="432" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="589" fillId="0" borderId="433" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="590" fillId="0" borderId="434" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="591" fillId="0" borderId="435" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="592" fillId="0" borderId="436" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="593" fillId="0" borderId="437" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="594" fillId="0" borderId="438" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="595" fillId="0" borderId="439" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="596" fillId="0" borderId="440" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="597" fillId="0" borderId="441" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7837,31 +8079,31 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="605" fillId="0" borderId="449" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="606" fillId="0" borderId="450" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="607" fillId="0" borderId="451" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="608" fillId="0" borderId="452" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="606" fillId="0" borderId="450" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="607" fillId="0" borderId="451" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="608" fillId="0" borderId="452" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="0" fontId="609" fillId="0" borderId="453" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="610" fillId="0" borderId="454" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="611" fillId="0" borderId="455" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="612" fillId="0" borderId="456" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7869,15 +8111,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="613" fillId="0" borderId="457" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="614" fillId="0" borderId="458" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="615" fillId="0" borderId="459" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="616" fillId="0" borderId="460" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -7889,82 +8131,170 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="618" fillId="0" borderId="462" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="619" fillId="0" borderId="463" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="620" fillId="0" borderId="464" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="621" fillId="0" borderId="465" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="622" fillId="0" borderId="466" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="623" fillId="0" borderId="467" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="624" fillId="0" borderId="468" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="625" fillId="0" borderId="469" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="626" fillId="0" borderId="470" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="627" fillId="0" borderId="471" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="628" fillId="0" borderId="472" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="629" fillId="0" borderId="473" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="630" fillId="0" borderId="474" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="631" fillId="0" borderId="475" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="632" fillId="0" borderId="476" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="633" fillId="0" borderId="477" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="634" fillId="0" borderId="478" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="635" fillId="0" borderId="479" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="636" fillId="0" borderId="480" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="637" fillId="0" borderId="481" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="638" fillId="0" borderId="482" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="639" fillId="0" borderId="483" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="640" fillId="0" borderId="484" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="619" fillId="0" borderId="463" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="641" fillId="0" borderId="485" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="620" fillId="0" borderId="464" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="642" fillId="0" borderId="486" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="621" fillId="0" borderId="465" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="643" fillId="0" borderId="487" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="622" fillId="0" borderId="466" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="644" fillId="0" borderId="488" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="623" fillId="0" borderId="467" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="645" fillId="0" borderId="489" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="624" fillId="0" borderId="468" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="646" fillId="0" borderId="490" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="625" fillId="0" borderId="469" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="647" fillId="0" borderId="491" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="626" fillId="0" borderId="470" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="648" fillId="0" borderId="492" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="627" fillId="0" borderId="471" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="649" fillId="0" borderId="493" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="628" fillId="0" borderId="472" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="650" fillId="0" borderId="494" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="629" fillId="0" borderId="473" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="651" fillId="0" borderId="495" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="630" fillId="0" borderId="474" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="652" fillId="0" borderId="496" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="631" fillId="0" borderId="475" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="653" fillId="0" borderId="497" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="632" fillId="0" borderId="476" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="654" fillId="0" borderId="498" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="633" fillId="0" borderId="477" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="655" fillId="0" borderId="499" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="634" fillId="0" borderId="478" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="656" fillId="0" borderId="500" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="635" fillId="0" borderId="479" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="657" fillId="0" borderId="501" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="637" fillId="0" borderId="480" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="659" fillId="0" borderId="502" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="639" fillId="0" borderId="481" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="661" fillId="0" borderId="503" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7988,87 +8318,87 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="E1" s="36" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="84" t="s">
+      <c r="B2" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="63" t="s">
+      <c r="D2" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="76" t="s">
+      <c r="E2" s="80" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="69" t="s">
+      <c r="C3" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="70" t="s">
+      <c r="D3" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="77" t="s">
+      <c r="E3" s="81" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="86" t="s">
+      <c r="B4" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="88" t="s">
+      <c r="C4" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="89" t="s">
+      <c r="D4" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="90" t="s">
+      <c r="E4" s="94" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="87" t="s">
+      <c r="B5" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="91" t="s">
+      <c r="C5" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="92" t="s">
+      <c r="D5" s="96" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="93" t="s">
+      <c r="E5" s="97" t="s">
         <v>12</v>
       </c>
     </row>
@@ -8085,148 +8415,148 @@
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="95" customWidth="true"/>
-    <col min="2" max="2" width="16.7109375" style="96" customWidth="true"/>
-    <col min="3" max="3" width="8.7109375" style="97" customWidth="true"/>
-    <col min="6" max="6" width="8.7109375" style="98" customWidth="true"/>
-    <col min="4" max="4" width="16.7109375" style="99" customWidth="true"/>
-    <col min="7" max="7" width="16.7109375" style="100" customWidth="true"/>
-    <col min="5" max="5" width="8.7109375" style="101" customWidth="true"/>
-    <col min="8" max="8" width="8.7109375" style="102" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="99" customWidth="true"/>
+    <col min="2" max="2" width="16.7109375" style="100" customWidth="true"/>
+    <col min="3" max="3" width="8.7109375" style="101" customWidth="true"/>
+    <col min="6" max="6" width="8.7109375" style="102" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="103" customWidth="true"/>
+    <col min="7" max="7" width="16.7109375" style="104" customWidth="true"/>
+    <col min="5" max="5" width="8.7109375" style="105" customWidth="true"/>
+    <col min="8" max="8" width="8.7109375" style="106" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="94" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="154" t="s">
+    <row r="1" s="98" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="162" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="143" t="s">
+      <c r="B1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="143" t="s">
+      <c r="C1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="143" t="s">
+      <c r="D1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="143" t="s">
+      <c r="E1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="143" t="s">
+      <c r="F1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="143" t="s">
+      <c r="G1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="143" t="s">
+      <c r="H1" s="151" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="111" t="s">
+      <c r="A2" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="227" t="s">
+      <c r="B2" s="235" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="193" t="s">
+      <c r="C2" s="201" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="202" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="195" t="s">
+      <c r="E2" s="203" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="196" t="s">
+      <c r="F2" s="204" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="197" t="s">
+      <c r="G2" s="205" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="219" t="s">
+      <c r="H2" s="227" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="119" t="s">
+      <c r="A3" s="127" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="228" t="s">
+      <c r="B3" s="236" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="206" t="s">
+      <c r="C3" s="214" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="207" t="s">
+      <c r="D3" s="215" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="208" t="s">
+      <c r="E3" s="216" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="209" t="s">
+      <c r="F3" s="217" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="210" t="s">
+      <c r="G3" s="218" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="220" t="s">
+      <c r="H3" s="228" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="127" t="s">
+      <c r="A4" s="135" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="229" t="s">
+      <c r="B4" s="237" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="238" t="s">
+      <c r="C4" s="246" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="239" t="s">
+      <c r="D4" s="247" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="240" t="s">
+      <c r="E4" s="248" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="241" t="s">
+      <c r="F4" s="249" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="242" t="s">
+      <c r="G4" s="250" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="243" t="s">
+      <c r="H4" s="251" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="135" t="s">
+      <c r="A5" s="143" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="231" t="s">
+      <c r="B5" s="239" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="244" t="s">
+      <c r="C5" s="252" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="245" t="s">
+      <c r="D5" s="253" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="246" t="s">
+      <c r="E5" s="254" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="247" t="s">
+      <c r="F5" s="255" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="248" t="s">
+      <c r="G5" s="256" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="249" t="s">
+      <c r="H5" s="257" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="254" t="s">
+      <c r="B6" s="262" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="0"/>
@@ -8251,95 +8581,95 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="256" customWidth="true"/>
-    <col min="2" max="2" width="13.7109375" style="257" customWidth="true"/>
-    <col min="3" max="3" width="13.7109375" style="258" customWidth="true"/>
-    <col min="4" max="4" width="16.7109375" style="259" customWidth="true"/>
-    <col min="5" max="5" width="8.7109375" style="260" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="264" customWidth="true"/>
+    <col min="2" max="2" width="13.7109375" style="265" customWidth="true"/>
+    <col min="3" max="3" width="13.7109375" style="266" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="267" customWidth="true"/>
+    <col min="5" max="5" width="8.7109375" style="268" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="255" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="294" t="s">
+    <row r="1" s="263" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="306" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="286" t="s">
+      <c r="B1" s="298" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="286" t="s">
+      <c r="C1" s="298" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="286" t="s">
+      <c r="D1" s="298" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="286" t="s">
+      <c r="E1" s="298" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="266" t="s">
+      <c r="A2" s="278" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="338" t="s">
+      <c r="B2" s="350" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="316" t="s">
+      <c r="C2" s="328" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="317" t="s">
+      <c r="D2" s="329" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="330" t="s">
+      <c r="E2" s="342" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="271" t="s">
+      <c r="A3" s="283" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="339" t="s">
+      <c r="B3" s="351" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="323" t="s">
+      <c r="C3" s="335" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="324" t="s">
+      <c r="D3" s="336" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="331" t="s">
+      <c r="E3" s="343" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="276" t="s">
+      <c r="A4" s="288" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="340" t="s">
+      <c r="B4" s="352" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="342" t="s">
+      <c r="C4" s="354" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="343" t="s">
+      <c r="D4" s="355" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="344" t="s">
+      <c r="E4" s="356" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="281" t="s">
+      <c r="A5" s="293" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="341" t="s">
+      <c r="B5" s="353" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="345" t="s">
+      <c r="C5" s="357" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="346" t="s">
+      <c r="D5" s="358" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="347" t="s">
+      <c r="E5" s="359" t="s">
         <v>12</v>
       </c>
     </row>
@@ -8356,151 +8686,151 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="349" customWidth="true"/>
-    <col min="2" max="2" width="28.7109375" style="350" customWidth="true"/>
-    <col min="3" max="3" width="8.7109375" style="351" customWidth="true"/>
-    <col min="4" max="4" width="16.7109375" style="352" customWidth="true"/>
-    <col min="5" max="5" width="8.7109375" style="353" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="361" customWidth="true"/>
+    <col min="2" max="2" width="28.7109375" style="362" customWidth="true"/>
+    <col min="3" max="3" width="8.7109375" style="363" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="364" customWidth="true"/>
+    <col min="5" max="5" width="8.7109375" style="365" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="348" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="402" t="s">
+    <row r="1" s="360" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="424" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="394" t="s">
+      <c r="B1" s="416" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="394" t="s">
+      <c r="C1" s="416" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="394" t="s">
+      <c r="D1" s="416" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="394" t="s">
+      <c r="E1" s="416" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="359" t="s">
+      <c r="A2" s="381" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="455" t="s">
+      <c r="B2" s="477" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="427" t="s">
+      <c r="C2" s="449" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="428" t="s">
+      <c r="D2" s="450" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="441" t="s">
+      <c r="E2" s="463" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="364" t="s">
+      <c r="A3" s="386" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="456" t="s">
+      <c r="B3" s="478" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="434" t="s">
+      <c r="C3" s="456" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="435" t="s">
+      <c r="D3" s="457" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="442" t="s">
+      <c r="E3" s="464" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="369" t="s">
+      <c r="A4" s="391" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="457" t="s">
+      <c r="B4" s="479" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="462" t="s">
+      <c r="C4" s="484" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="463" t="s">
+      <c r="D4" s="485" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="464" t="s">
+      <c r="E4" s="486" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="374" t="s">
+      <c r="A5" s="396" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="458" t="s">
+      <c r="B5" s="480" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="465" t="s">
+      <c r="C5" s="487" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="466" t="s">
+      <c r="D5" s="488" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="467" t="s">
+      <c r="E5" s="489" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="379" t="s">
+      <c r="A6" s="401" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="459" t="s">
+      <c r="B6" s="481" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="468" t="s">
+      <c r="C6" s="490" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="469" t="s">
+      <c r="D6" s="491" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="470" t="s">
+      <c r="E6" s="492" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="384" t="s">
+      <c r="A7" s="406" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="460" t="s">
+      <c r="B7" s="482" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="471" t="s">
+      <c r="C7" s="493" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="472" t="s">
+      <c r="D7" s="494" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="473" t="s">
+      <c r="E7" s="495" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="389" t="s">
+      <c r="A8" s="411" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="461" t="s">
+      <c r="B8" s="483" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="474" t="s">
+      <c r="C8" s="496" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="475" t="s">
+      <c r="D8" s="497" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="476" t="s">
+      <c r="E8" s="498" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="481" t="s">
+      <c r="B9" s="503" t="s">
         <v>39</v>
       </c>
       <c r="C9" s="0"/>

</xml_diff>